<commit_message>
Chap 8, Ex 18 and summary 8.1~8.2
</commit_message>
<xml_diff>
--- a/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
+++ b/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_387CDADADA3AA9B66CFD4D18C5A051F2DB1993B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD127417-EB1F-44FA-86AD-8ABB4806EFE2}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_387CDADADA3AA9B66CFD4D18C5A051F2DB1993B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E470017-5F79-4A53-B753-977DB9F9A4BF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="481">
   <si>
     <t>Order</t>
   </si>
@@ -1487,7 +1487,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -1569,13 +1569,13 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -1593,10 +1593,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1642,6 +1642,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1950,15 +1954,21 @@
       </c>
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="10"/>
+      <c r="L2" s="11">
+        <v>46273</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>233</v>
+      </c>
       <c r="N2" s="10"/>
       <c r="O2" s="10"/>
-      <c r="P2" s="11" t="str">
+      <c r="P2" s="11">
         <f>IF(AND($L2&lt;&gt;"",$M2&lt;&gt;""),$L2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
-      </c>
-      <c r="Q2" s="11"/>
+        <v>46275</v>
+      </c>
+      <c r="Q2" s="11">
+        <v>46278</v>
+      </c>
       <c r="R2" s="10"/>
       <c r="S2" s="10"/>
       <c r="T2" s="10" t="s">
@@ -2039,7 +2049,9 @@
         <f>IF(AND($L4&lt;&gt;"",$M4&lt;&gt;""),$L4+VLOOKUP($M4,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
         <v>46278</v>
       </c>
-      <c r="Q4" s="11"/>
+      <c r="Q4" s="11">
+        <v>46278</v>
+      </c>
       <c r="R4" s="10"/>
       <c r="S4" s="10"/>
       <c r="T4" s="10" t="s">
@@ -2115,13 +2127,17 @@
       </c>
       <c r="J6" s="11"/>
       <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="10"/>
+      <c r="L6" s="11">
+        <v>46278</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>236</v>
+      </c>
       <c r="N6" s="10"/>
       <c r="O6" s="10"/>
-      <c r="P6" s="11" t="str">
+      <c r="P6" s="11">
         <f>IF(AND($L6&lt;&gt;"",$M6&lt;&gt;""),$L6+VLOOKUP($M6,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46280</v>
       </c>
       <c r="Q6" s="11"/>
       <c r="R6" s="10"/>
@@ -3636,7 +3652,7 @@
       </c>
       <c r="B7" s="8">
         <f>COUNT('Master Schedule'!L2:L43)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">

</xml_diff>

<commit_message>
Chap 8, Ex 8
</commit_message>
<xml_diff>
--- a/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
+++ b/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_387CDADADA3AA9B66CFD4D18C5A051F2DB1993B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E470017-5F79-4A53-B753-977DB9F9A4BF}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_387CDADADA3AA9B66CFD4D18C5A051F2DB1993B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{912218EE-3BC4-4846-85B8-40082DF7C3B9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2040" yWindow="2220" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="481">
   <si>
     <t>Order</t>
   </si>
@@ -2170,13 +2170,17 @@
       </c>
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="6"/>
+      <c r="L7" s="12">
+        <v>46279</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>233</v>
+      </c>
       <c r="N7" s="6"/>
       <c r="O7" s="6"/>
-      <c r="P7" s="12" t="str">
+      <c r="P7" s="12">
         <f>IF(AND($L7&lt;&gt;"",$M7&lt;&gt;""),$L7+VLOOKUP($M7,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46281</v>
       </c>
       <c r="Q7" s="12"/>
       <c r="R7" s="6"/>
@@ -2209,13 +2213,17 @@
       </c>
       <c r="J8" s="11"/>
       <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="10"/>
+      <c r="L8" s="11">
+        <v>46279</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>233</v>
+      </c>
       <c r="N8" s="10"/>
       <c r="O8" s="10"/>
-      <c r="P8" s="11" t="str">
+      <c r="P8" s="11">
         <f>IF(AND($L8&lt;&gt;"",$M8&lt;&gt;""),$L8+VLOOKUP($M8,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46281</v>
       </c>
       <c r="Q8" s="11"/>
       <c r="R8" s="10"/>
@@ -3652,7 +3660,7 @@
       </c>
       <c r="B7" s="8">
         <f>COUNT('Master Schedule'!L2:L43)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">
@@ -3671,7 +3679,7 @@
       </c>
       <c r="B8" s="8">
         <f ca="1">COUNTIFS('Master Schedule'!P2:P43,"&lt;="&amp;TODAY(),'Master Schedule'!P2:P43,"&gt;0",'Master Schedule'!Q2:Q43,"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6" t="s">

</xml_diff>

<commit_message>
Chap 8, Ex 1, 7
</commit_message>
<xml_diff>
--- a/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
+++ b/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_0EA98B02D5D38FBAA81C65D3315416646CD29F91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EB51EAE-0243-4D72-89A1-395F2A947288}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_0EA98B02D5D38FBAA81C65D3315416646CD29F91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A6B4A0B-98E0-4D46-ADF3-B0CF224AB93B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="481">
   <si>
     <t>Order</t>
   </si>
@@ -1642,6 +1642,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1840,7 +1844,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T43"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -1862,7 +1866,7 @@
     <col min="20" max="20" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="27">
+    <row r="1" spans="1:20" ht="28">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1924,7 +1928,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="54">
+    <row r="2" spans="1:20" ht="56">
       <c r="A2" s="10">
         <v>1</v>
       </c>
@@ -1971,7 +1975,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="67.5">
+    <row r="3" spans="1:20" ht="70">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -2007,7 +2011,7 @@
       <c r="S3" s="6"/>
       <c r="T3" s="6"/>
     </row>
-    <row r="4" spans="1:20" ht="40.5">
+    <row r="4" spans="1:20" ht="42">
       <c r="A4" s="10">
         <v>3</v>
       </c>
@@ -2054,7 +2058,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="40.5">
+    <row r="5" spans="1:20" ht="42">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -2099,7 +2103,7 @@
       <c r="S5" s="6"/>
       <c r="T5" s="6"/>
     </row>
-    <row r="6" spans="1:20" ht="40.5">
+    <row r="6" spans="1:20" ht="42">
       <c r="A6" s="10">
         <v>5</v>
       </c>
@@ -2144,7 +2148,7 @@
       <c r="S6" s="10"/>
       <c r="T6" s="10"/>
     </row>
-    <row r="7" spans="1:20" ht="27">
+    <row r="7" spans="1:20" ht="28">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -2189,7 +2193,7 @@
       <c r="S7" s="6"/>
       <c r="T7" s="6"/>
     </row>
-    <row r="8" spans="1:20" ht="27">
+    <row r="8" spans="1:20" ht="28">
       <c r="A8" s="10">
         <v>7</v>
       </c>
@@ -2232,7 +2236,7 @@
       <c r="S8" s="10"/>
       <c r="T8" s="10"/>
     </row>
-    <row r="9" spans="1:20" ht="40.5">
+    <row r="9" spans="1:20" ht="42">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -2275,7 +2279,7 @@
       <c r="S9" s="6"/>
       <c r="T9" s="6"/>
     </row>
-    <row r="10" spans="1:20" ht="67.5">
+    <row r="10" spans="1:20" ht="70">
       <c r="A10" s="10">
         <v>9</v>
       </c>
@@ -2313,7 +2317,7 @@
       <c r="S10" s="10"/>
       <c r="T10" s="10"/>
     </row>
-    <row r="11" spans="1:20" ht="40.5">
+    <row r="11" spans="1:20" ht="42">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -2356,7 +2360,7 @@
       <c r="S11" s="6"/>
       <c r="T11" s="6"/>
     </row>
-    <row r="12" spans="1:20" ht="27">
+    <row r="12" spans="1:20" ht="28">
       <c r="A12" s="10">
         <v>11</v>
       </c>
@@ -2399,7 +2403,7 @@
       <c r="S12" s="10"/>
       <c r="T12" s="10"/>
     </row>
-    <row r="13" spans="1:20" ht="54">
+    <row r="13" spans="1:20" ht="56">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -2435,7 +2439,7 @@
       <c r="S13" s="6"/>
       <c r="T13" s="6"/>
     </row>
-    <row r="14" spans="1:20" ht="67.5">
+    <row r="14" spans="1:20" ht="70">
       <c r="A14" s="10">
         <v>13</v>
       </c>
@@ -2471,7 +2475,7 @@
       <c r="S14" s="10"/>
       <c r="T14" s="10"/>
     </row>
-    <row r="15" spans="1:20" ht="54">
+    <row r="15" spans="1:20" ht="56">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2514,7 +2518,7 @@
       <c r="S15" s="6"/>
       <c r="T15" s="6"/>
     </row>
-    <row r="16" spans="1:20" ht="54">
+    <row r="16" spans="1:20" ht="56">
       <c r="A16" s="10">
         <v>15</v>
       </c>
@@ -2550,7 +2554,7 @@
       <c r="S16" s="10"/>
       <c r="T16" s="10"/>
     </row>
-    <row r="17" spans="1:20" ht="27">
+    <row r="17" spans="1:20" ht="28">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2576,20 +2580,24 @@
       </c>
       <c r="J17" s="12"/>
       <c r="K17" s="12"/>
-      <c r="L17" s="12"/>
-      <c r="M17" s="6"/>
+      <c r="L17" s="12">
+        <v>46292</v>
+      </c>
+      <c r="M17" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="N17" s="6"/>
       <c r="O17" s="6"/>
-      <c r="P17" s="12" t="str">
+      <c r="P17" s="12">
         <f>IF(AND($L17&lt;&gt;"",$M17&lt;&gt;""),$L17+VLOOKUP($M17,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46294</v>
       </c>
       <c r="Q17" s="12"/>
       <c r="R17" s="6"/>
       <c r="S17" s="6"/>
       <c r="T17" s="6"/>
     </row>
-    <row r="18" spans="1:20" ht="27">
+    <row r="18" spans="1:20" ht="28">
       <c r="A18" s="10">
         <v>17</v>
       </c>
@@ -2628,7 +2636,7 @@
       <c r="S18" s="10"/>
       <c r="T18" s="10"/>
     </row>
-    <row r="19" spans="1:20" ht="67.5">
+    <row r="19" spans="1:20" ht="70">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2664,7 +2672,7 @@
       <c r="S19" s="6"/>
       <c r="T19" s="6"/>
     </row>
-    <row r="20" spans="1:20" ht="40.5">
+    <row r="20" spans="1:20" ht="42">
       <c r="A20" s="10">
         <v>19</v>
       </c>
@@ -2703,7 +2711,7 @@
       <c r="S20" s="10"/>
       <c r="T20" s="10"/>
     </row>
-    <row r="21" spans="1:20" ht="40.5">
+    <row r="21" spans="1:20" ht="42">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2781,7 +2789,7 @@
       <c r="S22" s="10"/>
       <c r="T22" s="10"/>
     </row>
-    <row r="23" spans="1:20" ht="40.5">
+    <row r="23" spans="1:20" ht="42">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2820,7 +2828,7 @@
       <c r="S23" s="6"/>
       <c r="T23" s="6"/>
     </row>
-    <row r="24" spans="1:20" ht="54">
+    <row r="24" spans="1:20" ht="56">
       <c r="A24" s="10">
         <v>23</v>
       </c>
@@ -2854,7 +2862,7 @@
       <c r="S24" s="10"/>
       <c r="T24" s="10"/>
     </row>
-    <row r="25" spans="1:20" ht="40.5">
+    <row r="25" spans="1:20" ht="42">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -2893,7 +2901,7 @@
       <c r="S25" s="6"/>
       <c r="T25" s="6"/>
     </row>
-    <row r="26" spans="1:20" ht="40.5">
+    <row r="26" spans="1:20" ht="42">
       <c r="A26" s="10">
         <v>25</v>
       </c>
@@ -2932,7 +2940,7 @@
       <c r="S26" s="10"/>
       <c r="T26" s="10"/>
     </row>
-    <row r="27" spans="1:20" ht="67.5">
+    <row r="27" spans="1:20" ht="70">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -2966,7 +2974,7 @@
       <c r="S27" s="6"/>
       <c r="T27" s="6"/>
     </row>
-    <row r="28" spans="1:20" ht="40.5">
+    <row r="28" spans="1:20" ht="42">
       <c r="A28" s="10">
         <v>27</v>
       </c>
@@ -3005,7 +3013,7 @@
       <c r="S28" s="10"/>
       <c r="T28" s="10"/>
     </row>
-    <row r="29" spans="1:20" ht="67.5">
+    <row r="29" spans="1:20" ht="70">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -3044,7 +3052,7 @@
       <c r="S29" s="6"/>
       <c r="T29" s="6"/>
     </row>
-    <row r="30" spans="1:20" ht="54">
+    <row r="30" spans="1:20" ht="56">
       <c r="A30" s="10">
         <v>29</v>
       </c>
@@ -3080,7 +3088,7 @@
       <c r="S30" s="10"/>
       <c r="T30" s="10"/>
     </row>
-    <row r="31" spans="1:20" ht="54">
+    <row r="31" spans="1:20" ht="56">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -3114,7 +3122,7 @@
       <c r="S31" s="6"/>
       <c r="T31" s="6"/>
     </row>
-    <row r="32" spans="1:20" ht="67.5">
+    <row r="32" spans="1:20" ht="70">
       <c r="A32" s="10">
         <v>31</v>
       </c>
@@ -3150,7 +3158,7 @@
       <c r="S32" s="10"/>
       <c r="T32" s="10"/>
     </row>
-    <row r="33" spans="1:20" ht="27">
+    <row r="33" spans="1:20" ht="28">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -3189,7 +3197,7 @@
       <c r="S33" s="6"/>
       <c r="T33" s="6"/>
     </row>
-    <row r="34" spans="1:20" ht="40.5">
+    <row r="34" spans="1:20" ht="42">
       <c r="A34" s="10">
         <v>33</v>
       </c>
@@ -3228,7 +3236,7 @@
       <c r="S34" s="10"/>
       <c r="T34" s="10"/>
     </row>
-    <row r="35" spans="1:20" ht="81">
+    <row r="35" spans="1:20" ht="84">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -3340,7 +3348,7 @@
       <c r="S37" s="6"/>
       <c r="T37" s="6"/>
     </row>
-    <row r="38" spans="1:20" ht="27">
+    <row r="38" spans="1:20" ht="28">
       <c r="A38" s="10">
         <v>37</v>
       </c>
@@ -3379,7 +3387,7 @@
       <c r="S38" s="10"/>
       <c r="T38" s="10"/>
     </row>
-    <row r="39" spans="1:20" ht="54">
+    <row r="39" spans="1:20" ht="56">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3418,7 +3426,7 @@
       <c r="S39" s="6"/>
       <c r="T39" s="6"/>
     </row>
-    <row r="40" spans="1:20" ht="54">
+    <row r="40" spans="1:20" ht="56">
       <c r="A40" s="10">
         <v>39</v>
       </c>
@@ -3452,7 +3460,7 @@
       <c r="S40" s="10"/>
       <c r="T40" s="10"/>
     </row>
-    <row r="41" spans="1:20" ht="67.5">
+    <row r="41" spans="1:20" ht="70">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3488,7 +3496,7 @@
       <c r="S41" s="6"/>
       <c r="T41" s="6"/>
     </row>
-    <row r="42" spans="1:20" ht="54">
+    <row r="42" spans="1:20" ht="56">
       <c r="A42" s="10">
         <v>41</v>
       </c>
@@ -3522,7 +3530,7 @@
       <c r="S42" s="10"/>
       <c r="T42" s="10"/>
     </row>
-    <row r="43" spans="1:20" ht="40.5">
+    <row r="43" spans="1:20" ht="42">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3584,7 +3592,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -3594,7 +3602,7 @@
     <col min="6" max="6" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75">
+    <row r="1" spans="1:6" ht="17.5">
       <c r="A1" s="13" t="s">
         <v>176</v>
       </c>
@@ -3640,7 +3648,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="27">
+    <row r="5" spans="1:6" ht="28">
       <c r="A5" s="6" t="s">
         <v>183</v>
       </c>
@@ -3659,7 +3667,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="27">
+    <row r="6" spans="1:6" ht="28">
       <c r="A6" s="6" t="s">
         <v>186</v>
       </c>
@@ -3678,13 +3686,13 @@
         <v>189</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="27">
+    <row r="7" spans="1:6" ht="28">
       <c r="A7" s="6" t="s">
         <v>190</v>
       </c>
       <c r="B7" s="8">
         <f>COUNT('Master Schedule'!L2:L43)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">
@@ -3697,13 +3705,13 @@
         <v>192</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="27">
+    <row r="8" spans="1:6" ht="28">
       <c r="A8" s="6" t="s">
         <v>193</v>
       </c>
       <c r="B8" s="8">
         <f ca="1">COUNTIFS('Master Schedule'!P2:P43,"&lt;="&amp;TODAY(),'Master Schedule'!P2:P43,"&gt;0",'Master Schedule'!Q2:Q43,"")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6" t="s">
@@ -3716,7 +3724,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="27">
+    <row r="9" spans="1:6" ht="28">
       <c r="A9" s="6" t="s">
         <v>196</v>
       </c>
@@ -3761,7 +3769,7 @@
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
     </row>
-    <row r="13" spans="1:6" ht="27">
+    <row r="13" spans="1:6" ht="28">
       <c r="A13" s="6" t="s">
         <v>200</v>
       </c>
@@ -3775,7 +3783,7 @@
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
     </row>
-    <row r="14" spans="1:6" ht="27">
+    <row r="14" spans="1:6" ht="28">
       <c r="A14" s="6" t="s">
         <v>203</v>
       </c>
@@ -3803,7 +3811,7 @@
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
     </row>
-    <row r="16" spans="1:6" ht="40.5">
+    <row r="16" spans="1:6" ht="42">
       <c r="A16" s="6" t="s">
         <v>209</v>
       </c>
@@ -3831,7 +3839,7 @@
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
     </row>
-    <row r="18" spans="1:6" ht="27">
+    <row r="18" spans="1:6" ht="28">
       <c r="A18" s="6" t="s">
         <v>215</v>
       </c>
@@ -3863,7 +3871,7 @@
       <c r="E20" s="15"/>
       <c r="F20" s="15"/>
     </row>
-    <row r="21" spans="1:6" ht="40.5">
+    <row r="21" spans="1:6" ht="42">
       <c r="A21" s="6" t="s">
         <v>32</v>
       </c>
@@ -3877,7 +3885,7 @@
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
     </row>
-    <row r="22" spans="1:6" ht="40.5">
+    <row r="22" spans="1:6" ht="42">
       <c r="A22" s="6" t="s">
         <v>121</v>
       </c>
@@ -3891,7 +3899,7 @@
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
     </row>
-    <row r="23" spans="1:6" ht="27">
+    <row r="23" spans="1:6" ht="28">
       <c r="A23" s="6" t="s">
         <v>155</v>
       </c>
@@ -3920,7 +3928,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -3928,7 +3936,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27">
+    <row r="1" spans="1:4" ht="28">
       <c r="A1" s="1" t="s">
         <v>225</v>
       </c>
@@ -3942,7 +3950,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="40.5">
+    <row r="2" spans="1:4" ht="42">
       <c r="A2" s="2" t="s">
         <v>229</v>
       </c>
@@ -3956,7 +3964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="27">
+    <row r="3" spans="1:4" ht="28">
       <c r="A3" s="4" t="s">
         <v>232</v>
       </c>
@@ -3970,7 +3978,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="27">
+    <row r="4" spans="1:4" ht="28">
       <c r="A4" s="2" t="s">
         <v>25</v>
       </c>
@@ -3984,7 +3992,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="27">
+    <row r="5" spans="1:4" ht="28">
       <c r="A5" s="4" t="s">
         <v>40</v>
       </c>
@@ -4016,7 +4024,7 @@
       </c>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:4" ht="27">
+    <row r="8" spans="1:4" ht="28">
       <c r="A8" s="2" t="s">
         <v>241</v>
       </c>
@@ -4028,7 +4036,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" ht="40.5">
+    <row r="9" spans="1:4" ht="42">
       <c r="A9" s="4" t="s">
         <v>244</v>
       </c>
@@ -4040,7 +4048,7 @@
       </c>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4" ht="40.5">
+    <row r="10" spans="1:4" ht="42">
       <c r="A10" s="2" t="s">
         <v>247</v>
       </c>
@@ -4052,7 +4060,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" ht="40.5">
+    <row r="11" spans="1:4" ht="42">
       <c r="A11" s="4" t="s">
         <v>250</v>
       </c>
@@ -4064,7 +4072,7 @@
       </c>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" ht="40.5">
+    <row r="12" spans="1:4" ht="42">
       <c r="A12" s="2" t="s">
         <v>253</v>
       </c>
@@ -4076,7 +4084,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" ht="27">
+    <row r="13" spans="1:4" ht="28">
       <c r="A13" s="4" t="s">
         <v>256</v>
       </c>
@@ -4088,7 +4096,7 @@
       </c>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" ht="40.5">
+    <row r="14" spans="1:4" ht="42">
       <c r="A14" s="2" t="s">
         <v>259</v>
       </c>
@@ -4100,7 +4108,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:4" ht="40.5">
+    <row r="15" spans="1:4" ht="42">
       <c r="A15" s="4" t="s">
         <v>262</v>
       </c>
@@ -4112,7 +4120,7 @@
       </c>
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:4" ht="40.5">
+    <row r="16" spans="1:4" ht="42">
       <c r="A16" s="2" t="s">
         <v>265</v>
       </c>
@@ -4124,7 +4132,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" ht="40.5">
+    <row r="17" spans="1:4" ht="42">
       <c r="A17" s="4" t="s">
         <v>268</v>
       </c>
@@ -4145,7 +4153,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -4158,7 +4166,7 @@
     <col min="9" max="9" width="46" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.75">
+    <row r="1" spans="1:9" ht="17.5">
       <c r="A1" s="16" t="s">
         <v>271</v>
       </c>
@@ -4184,7 +4192,7 @@
       <c r="H2" s="17"/>
       <c r="I2" s="17"/>
     </row>
-    <row r="3" spans="1:9" ht="27">
+    <row r="3" spans="1:9" ht="28">
       <c r="A3" s="1" t="s">
         <v>273</v>
       </c>
@@ -4213,7 +4221,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="27">
+    <row r="4" spans="1:9" ht="28">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -4242,7 +4250,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="27">
+    <row r="5" spans="1:9" ht="28">
       <c r="A5" s="4">
         <v>2</v>
       </c>
@@ -4271,7 +4279,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="40.5">
+    <row r="6" spans="1:9" ht="42">
       <c r="A6" s="2">
         <v>3</v>
       </c>
@@ -4300,7 +4308,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="40.5">
+    <row r="7" spans="1:9" ht="42">
       <c r="A7" s="4">
         <v>4</v>
       </c>
@@ -4329,7 +4337,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="27">
+    <row r="8" spans="1:9" ht="28">
       <c r="A8" s="2">
         <v>5</v>
       </c>
@@ -4358,7 +4366,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="27">
+    <row r="9" spans="1:9" ht="28">
       <c r="A9" s="4">
         <v>6</v>
       </c>
@@ -4474,7 +4482,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="27">
+    <row r="13" spans="1:9" ht="28">
       <c r="A13" s="4">
         <v>10</v>
       </c>
@@ -4532,7 +4540,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="27">
+    <row r="15" spans="1:9" ht="28">
       <c r="A15" s="4">
         <v>12</v>
       </c>
@@ -4561,7 +4569,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="40.5">
+    <row r="16" spans="1:9" ht="42">
       <c r="A16" s="2">
         <v>13</v>
       </c>
@@ -4590,7 +4598,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="27">
+    <row r="17" spans="1:9" ht="28">
       <c r="A17" s="4">
         <v>14</v>
       </c>
@@ -4619,7 +4627,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="27">
+    <row r="18" spans="1:9" ht="28">
       <c r="A18" s="2">
         <v>15</v>
       </c>
@@ -4648,7 +4656,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="27">
+    <row r="19" spans="1:9" ht="28">
       <c r="A19" s="4">
         <v>16</v>
       </c>
@@ -4677,7 +4685,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="27">
+    <row r="20" spans="1:9" ht="28">
       <c r="A20" s="2">
         <v>17</v>
       </c>
@@ -4764,7 +4772,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="27">
+    <row r="23" spans="1:9" ht="28">
       <c r="A23" s="4">
         <v>20</v>
       </c>
@@ -4793,7 +4801,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="27">
+    <row r="24" spans="1:9" ht="28">
       <c r="A24" s="2">
         <v>21</v>
       </c>
@@ -4851,7 +4859,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="27">
+    <row r="26" spans="1:9" ht="28">
       <c r="A26" s="2">
         <v>23</v>
       </c>
@@ -4880,7 +4888,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="27">
+    <row r="27" spans="1:9" ht="28">
       <c r="A27" s="4">
         <v>24</v>
       </c>
@@ -4909,7 +4917,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="27">
+    <row r="28" spans="1:9" ht="28">
       <c r="A28" s="2">
         <v>25</v>
       </c>
@@ -4996,7 +5004,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="27">
+    <row r="31" spans="1:9" ht="28">
       <c r="A31" s="4">
         <v>28</v>
       </c>
@@ -5054,7 +5062,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="27">
+    <row r="33" spans="1:9" ht="28">
       <c r="A33" s="4">
         <v>30</v>
       </c>
@@ -5083,7 +5091,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="27">
+    <row r="34" spans="1:9" ht="28">
       <c r="A34" s="2">
         <v>31</v>
       </c>
@@ -5141,7 +5149,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="27">
+    <row r="36" spans="1:9" ht="28">
       <c r="A36" s="2">
         <v>33</v>
       </c>
@@ -5199,7 +5207,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="27">
+    <row r="38" spans="1:9" ht="28">
       <c r="A38" s="2">
         <v>35</v>
       </c>
@@ -5228,7 +5236,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="27">
+    <row r="39" spans="1:9" ht="28">
       <c r="A39" s="4">
         <v>36</v>
       </c>
@@ -5270,7 +5278,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
@@ -5284,7 +5292,7 @@
     <col min="11" max="11" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75">
+    <row r="1" spans="1:11" ht="17.5">
       <c r="A1" s="16" t="s">
         <v>404</v>
       </c>
@@ -5314,7 +5322,7 @@
       <c r="J2" s="17"/>
       <c r="K2" s="17"/>
     </row>
-    <row r="3" spans="1:11" ht="27">
+    <row r="3" spans="1:11" ht="28">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -5349,7 +5357,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="67.5">
+    <row r="4" spans="1:11" ht="70">
       <c r="A4" s="2" t="s">
         <v>415</v>
       </c>
@@ -5378,7 +5386,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="54">
+    <row r="5" spans="1:11" ht="56">
       <c r="A5" s="4" t="s">
         <v>38</v>
       </c>
@@ -5405,7 +5413,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="54">
+    <row r="6" spans="1:11" ht="56">
       <c r="A6" s="2" t="s">
         <v>429</v>
       </c>
@@ -5430,7 +5438,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="40.5">
+    <row r="7" spans="1:11" ht="42">
       <c r="A7" s="4" t="s">
         <v>435</v>
       </c>
@@ -5453,7 +5461,7 @@
       <c r="J7" s="5"/>
       <c r="K7" s="4"/>
     </row>
-    <row r="8" spans="1:11" ht="40.5">
+    <row r="8" spans="1:11" ht="42">
       <c r="A8" s="2" t="s">
         <v>439</v>
       </c>
@@ -5480,7 +5488,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="54">
+    <row r="9" spans="1:11" ht="56">
       <c r="A9" s="4" t="s">
         <v>98</v>
       </c>
@@ -5507,7 +5515,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="54">
+    <row r="10" spans="1:11" ht="56">
       <c r="A10" s="2" t="s">
         <v>452</v>
       </c>
@@ -5530,7 +5538,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="40.5">
+    <row r="11" spans="1:11" ht="42">
       <c r="A11" s="4" t="s">
         <v>457</v>
       </c>
@@ -5557,7 +5565,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11" ht="40.5">
+    <row r="12" spans="1:11" ht="42">
       <c r="A12" s="2" t="s">
         <v>463</v>
       </c>
@@ -5582,7 +5590,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="40.5">
+    <row r="13" spans="1:11" ht="42">
       <c r="A13" s="4" t="s">
         <v>142</v>
       </c>
@@ -5607,7 +5615,7 @@
       <c r="J13" s="5"/>
       <c r="K13" s="4"/>
     </row>
-    <row r="14" spans="1:11" ht="40.5">
+    <row r="14" spans="1:11" ht="42">
       <c r="A14" s="2" t="s">
         <v>474</v>
       </c>

</xml_diff>

<commit_message>
Chap 8, Ex 33
</commit_message>
<xml_diff>
--- a/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
+++ b/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_0EA98B02D5D38FBAA81C65D3315416646CD29F91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A6B4A0B-98E0-4D46-ADF3-B0CF224AB93B}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_DE2EFB3A9D1E79C6859C80A3377C0E0772D29E3B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF23E7C9-3F0B-47DB-9547-EF99EC340627}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="481">
   <si>
     <t>Order</t>
   </si>
@@ -1642,10 +1642,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1844,7 +1840,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T43"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -1866,7 +1862,7 @@
     <col min="20" max="20" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="28">
+    <row r="1" spans="1:20" ht="27">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1928,7 +1924,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="56">
+    <row r="2" spans="1:20" ht="54">
       <c r="A2" s="10">
         <v>1</v>
       </c>
@@ -1975,7 +1971,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="70">
+    <row r="3" spans="1:20" ht="67.5">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -2011,7 +2007,7 @@
       <c r="S3" s="6"/>
       <c r="T3" s="6"/>
     </row>
-    <row r="4" spans="1:20" ht="42">
+    <row r="4" spans="1:20" ht="40.5">
       <c r="A4" s="10">
         <v>3</v>
       </c>
@@ -2058,7 +2054,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="42">
+    <row r="5" spans="1:20" ht="40.5">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -2103,7 +2099,7 @@
       <c r="S5" s="6"/>
       <c r="T5" s="6"/>
     </row>
-    <row r="6" spans="1:20" ht="42">
+    <row r="6" spans="1:20" ht="40.5">
       <c r="A6" s="10">
         <v>5</v>
       </c>
@@ -2148,7 +2144,7 @@
       <c r="S6" s="10"/>
       <c r="T6" s="10"/>
     </row>
-    <row r="7" spans="1:20" ht="28">
+    <row r="7" spans="1:20" ht="27">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -2193,7 +2189,7 @@
       <c r="S7" s="6"/>
       <c r="T7" s="6"/>
     </row>
-    <row r="8" spans="1:20" ht="28">
+    <row r="8" spans="1:20" ht="27">
       <c r="A8" s="10">
         <v>7</v>
       </c>
@@ -2236,7 +2232,7 @@
       <c r="S8" s="10"/>
       <c r="T8" s="10"/>
     </row>
-    <row r="9" spans="1:20" ht="42">
+    <row r="9" spans="1:20" ht="40.5">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -2279,7 +2275,7 @@
       <c r="S9" s="6"/>
       <c r="T9" s="6"/>
     </row>
-    <row r="10" spans="1:20" ht="70">
+    <row r="10" spans="1:20" ht="67.5">
       <c r="A10" s="10">
         <v>9</v>
       </c>
@@ -2317,7 +2313,7 @@
       <c r="S10" s="10"/>
       <c r="T10" s="10"/>
     </row>
-    <row r="11" spans="1:20" ht="42">
+    <row r="11" spans="1:20" ht="40.5">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -2360,7 +2356,7 @@
       <c r="S11" s="6"/>
       <c r="T11" s="6"/>
     </row>
-    <row r="12" spans="1:20" ht="28">
+    <row r="12" spans="1:20" ht="27">
       <c r="A12" s="10">
         <v>11</v>
       </c>
@@ -2403,7 +2399,7 @@
       <c r="S12" s="10"/>
       <c r="T12" s="10"/>
     </row>
-    <row r="13" spans="1:20" ht="56">
+    <row r="13" spans="1:20" ht="54">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -2439,7 +2435,7 @@
       <c r="S13" s="6"/>
       <c r="T13" s="6"/>
     </row>
-    <row r="14" spans="1:20" ht="70">
+    <row r="14" spans="1:20" ht="67.5">
       <c r="A14" s="10">
         <v>13</v>
       </c>
@@ -2475,7 +2471,7 @@
       <c r="S14" s="10"/>
       <c r="T14" s="10"/>
     </row>
-    <row r="15" spans="1:20" ht="56">
+    <row r="15" spans="1:20" ht="54">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2518,7 +2514,7 @@
       <c r="S15" s="6"/>
       <c r="T15" s="6"/>
     </row>
-    <row r="16" spans="1:20" ht="56">
+    <row r="16" spans="1:20" ht="54">
       <c r="A16" s="10">
         <v>15</v>
       </c>
@@ -2554,7 +2550,7 @@
       <c r="S16" s="10"/>
       <c r="T16" s="10"/>
     </row>
-    <row r="17" spans="1:20" ht="28">
+    <row r="17" spans="1:20" ht="27">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2597,7 +2593,7 @@
       <c r="S17" s="6"/>
       <c r="T17" s="6"/>
     </row>
-    <row r="18" spans="1:20" ht="28">
+    <row r="18" spans="1:20" ht="27">
       <c r="A18" s="10">
         <v>17</v>
       </c>
@@ -2623,20 +2619,24 @@
       </c>
       <c r="J18" s="11"/>
       <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="10"/>
+      <c r="L18" s="11">
+        <v>46292</v>
+      </c>
+      <c r="M18" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="N18" s="10"/>
       <c r="O18" s="10"/>
-      <c r="P18" s="11" t="str">
+      <c r="P18" s="11">
         <f>IF(AND($L18&lt;&gt;"",$M18&lt;&gt;""),$L18+VLOOKUP($M18,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46294</v>
       </c>
       <c r="Q18" s="11"/>
       <c r="R18" s="10"/>
       <c r="S18" s="10"/>
       <c r="T18" s="10"/>
     </row>
-    <row r="19" spans="1:20" ht="70">
+    <row r="19" spans="1:20" ht="67.5">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2672,7 +2672,7 @@
       <c r="S19" s="6"/>
       <c r="T19" s="6"/>
     </row>
-    <row r="20" spans="1:20" ht="42">
+    <row r="20" spans="1:20" ht="40.5">
       <c r="A20" s="10">
         <v>19</v>
       </c>
@@ -2698,20 +2698,24 @@
       </c>
       <c r="J20" s="11"/>
       <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="10"/>
+      <c r="L20" s="11">
+        <v>46299</v>
+      </c>
+      <c r="M20" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="N20" s="10"/>
       <c r="O20" s="10"/>
-      <c r="P20" s="11" t="str">
+      <c r="P20" s="11">
         <f>IF(AND($L20&lt;&gt;"",$M20&lt;&gt;""),$L20+VLOOKUP($M20,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46301</v>
       </c>
       <c r="Q20" s="11"/>
       <c r="R20" s="10"/>
       <c r="S20" s="10"/>
       <c r="T20" s="10"/>
     </row>
-    <row r="21" spans="1:20" ht="42">
+    <row r="21" spans="1:20" ht="40.5">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2789,7 +2793,7 @@
       <c r="S22" s="10"/>
       <c r="T22" s="10"/>
     </row>
-    <row r="23" spans="1:20" ht="42">
+    <row r="23" spans="1:20" ht="40.5">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2828,7 +2832,7 @@
       <c r="S23" s="6"/>
       <c r="T23" s="6"/>
     </row>
-    <row r="24" spans="1:20" ht="56">
+    <row r="24" spans="1:20" ht="54">
       <c r="A24" s="10">
         <v>23</v>
       </c>
@@ -2862,7 +2866,7 @@
       <c r="S24" s="10"/>
       <c r="T24" s="10"/>
     </row>
-    <row r="25" spans="1:20" ht="42">
+    <row r="25" spans="1:20" ht="40.5">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -2901,7 +2905,7 @@
       <c r="S25" s="6"/>
       <c r="T25" s="6"/>
     </row>
-    <row r="26" spans="1:20" ht="42">
+    <row r="26" spans="1:20" ht="40.5">
       <c r="A26" s="10">
         <v>25</v>
       </c>
@@ -2940,7 +2944,7 @@
       <c r="S26" s="10"/>
       <c r="T26" s="10"/>
     </row>
-    <row r="27" spans="1:20" ht="70">
+    <row r="27" spans="1:20" ht="67.5">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -2974,7 +2978,7 @@
       <c r="S27" s="6"/>
       <c r="T27" s="6"/>
     </row>
-    <row r="28" spans="1:20" ht="42">
+    <row r="28" spans="1:20" ht="40.5">
       <c r="A28" s="10">
         <v>27</v>
       </c>
@@ -3013,7 +3017,7 @@
       <c r="S28" s="10"/>
       <c r="T28" s="10"/>
     </row>
-    <row r="29" spans="1:20" ht="70">
+    <row r="29" spans="1:20" ht="67.5">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -3052,7 +3056,7 @@
       <c r="S29" s="6"/>
       <c r="T29" s="6"/>
     </row>
-    <row r="30" spans="1:20" ht="56">
+    <row r="30" spans="1:20" ht="54">
       <c r="A30" s="10">
         <v>29</v>
       </c>
@@ -3088,7 +3092,7 @@
       <c r="S30" s="10"/>
       <c r="T30" s="10"/>
     </row>
-    <row r="31" spans="1:20" ht="56">
+    <row r="31" spans="1:20" ht="54">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -3122,7 +3126,7 @@
       <c r="S31" s="6"/>
       <c r="T31" s="6"/>
     </row>
-    <row r="32" spans="1:20" ht="70">
+    <row r="32" spans="1:20" ht="67.5">
       <c r="A32" s="10">
         <v>31</v>
       </c>
@@ -3158,7 +3162,7 @@
       <c r="S32" s="10"/>
       <c r="T32" s="10"/>
     </row>
-    <row r="33" spans="1:20" ht="28">
+    <row r="33" spans="1:20" ht="27">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -3197,7 +3201,7 @@
       <c r="S33" s="6"/>
       <c r="T33" s="6"/>
     </row>
-    <row r="34" spans="1:20" ht="42">
+    <row r="34" spans="1:20" ht="40.5">
       <c r="A34" s="10">
         <v>33</v>
       </c>
@@ -3236,7 +3240,7 @@
       <c r="S34" s="10"/>
       <c r="T34" s="10"/>
     </row>
-    <row r="35" spans="1:20" ht="84">
+    <row r="35" spans="1:20" ht="81">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -3348,7 +3352,7 @@
       <c r="S37" s="6"/>
       <c r="T37" s="6"/>
     </row>
-    <row r="38" spans="1:20" ht="28">
+    <row r="38" spans="1:20" ht="27">
       <c r="A38" s="10">
         <v>37</v>
       </c>
@@ -3387,7 +3391,7 @@
       <c r="S38" s="10"/>
       <c r="T38" s="10"/>
     </row>
-    <row r="39" spans="1:20" ht="56">
+    <row r="39" spans="1:20" ht="54">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3426,7 +3430,7 @@
       <c r="S39" s="6"/>
       <c r="T39" s="6"/>
     </row>
-    <row r="40" spans="1:20" ht="56">
+    <row r="40" spans="1:20" ht="54">
       <c r="A40" s="10">
         <v>39</v>
       </c>
@@ -3460,7 +3464,7 @@
       <c r="S40" s="10"/>
       <c r="T40" s="10"/>
     </row>
-    <row r="41" spans="1:20" ht="70">
+    <row r="41" spans="1:20" ht="67.5">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3496,7 +3500,7 @@
       <c r="S41" s="6"/>
       <c r="T41" s="6"/>
     </row>
-    <row r="42" spans="1:20" ht="56">
+    <row r="42" spans="1:20" ht="54">
       <c r="A42" s="10">
         <v>41</v>
       </c>
@@ -3530,7 +3534,7 @@
       <c r="S42" s="10"/>
       <c r="T42" s="10"/>
     </row>
-    <row r="43" spans="1:20" ht="42">
+    <row r="43" spans="1:20" ht="40.5">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3592,7 +3596,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -3602,7 +3606,7 @@
     <col min="6" max="6" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.5">
+    <row r="1" spans="1:6" ht="18.75">
       <c r="A1" s="13" t="s">
         <v>176</v>
       </c>
@@ -3648,7 +3652,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="28">
+    <row r="5" spans="1:6" ht="27">
       <c r="A5" s="6" t="s">
         <v>183</v>
       </c>
@@ -3667,7 +3671,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="28">
+    <row r="6" spans="1:6" ht="27">
       <c r="A6" s="6" t="s">
         <v>186</v>
       </c>
@@ -3686,13 +3690,13 @@
         <v>189</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="28">
+    <row r="7" spans="1:6" ht="27">
       <c r="A7" s="6" t="s">
         <v>190</v>
       </c>
       <c r="B7" s="8">
         <f>COUNT('Master Schedule'!L2:L43)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">
@@ -3705,13 +3709,13 @@
         <v>192</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="28">
+    <row r="8" spans="1:6" ht="27">
       <c r="A8" s="6" t="s">
         <v>193</v>
       </c>
       <c r="B8" s="8">
         <f ca="1">COUNTIFS('Master Schedule'!P2:P43,"&lt;="&amp;TODAY(),'Master Schedule'!P2:P43,"&gt;0",'Master Schedule'!Q2:Q43,"")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6" t="s">
@@ -3724,7 +3728,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="28">
+    <row r="9" spans="1:6" ht="27">
       <c r="A9" s="6" t="s">
         <v>196</v>
       </c>
@@ -3769,7 +3773,7 @@
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
     </row>
-    <row r="13" spans="1:6" ht="28">
+    <row r="13" spans="1:6" ht="27">
       <c r="A13" s="6" t="s">
         <v>200</v>
       </c>
@@ -3783,7 +3787,7 @@
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
     </row>
-    <row r="14" spans="1:6" ht="28">
+    <row r="14" spans="1:6" ht="27">
       <c r="A14" s="6" t="s">
         <v>203</v>
       </c>
@@ -3811,7 +3815,7 @@
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
     </row>
-    <row r="16" spans="1:6" ht="42">
+    <row r="16" spans="1:6" ht="40.5">
       <c r="A16" s="6" t="s">
         <v>209</v>
       </c>
@@ -3839,7 +3843,7 @@
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
     </row>
-    <row r="18" spans="1:6" ht="28">
+    <row r="18" spans="1:6" ht="27">
       <c r="A18" s="6" t="s">
         <v>215</v>
       </c>
@@ -3871,7 +3875,7 @@
       <c r="E20" s="15"/>
       <c r="F20" s="15"/>
     </row>
-    <row r="21" spans="1:6" ht="42">
+    <row r="21" spans="1:6" ht="40.5">
       <c r="A21" s="6" t="s">
         <v>32</v>
       </c>
@@ -3885,7 +3889,7 @@
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
     </row>
-    <row r="22" spans="1:6" ht="42">
+    <row r="22" spans="1:6" ht="40.5">
       <c r="A22" s="6" t="s">
         <v>121</v>
       </c>
@@ -3899,7 +3903,7 @@
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
     </row>
-    <row r="23" spans="1:6" ht="28">
+    <row r="23" spans="1:6" ht="27">
       <c r="A23" s="6" t="s">
         <v>155</v>
       </c>
@@ -3928,7 +3932,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -3936,7 +3940,7 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28">
+    <row r="1" spans="1:4" ht="27">
       <c r="A1" s="1" t="s">
         <v>225</v>
       </c>
@@ -3950,7 +3954,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="42">
+    <row r="2" spans="1:4" ht="40.5">
       <c r="A2" s="2" t="s">
         <v>229</v>
       </c>
@@ -3964,7 +3968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28">
+    <row r="3" spans="1:4" ht="27">
       <c r="A3" s="4" t="s">
         <v>232</v>
       </c>
@@ -3978,7 +3982,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28">
+    <row r="4" spans="1:4" ht="27">
       <c r="A4" s="2" t="s">
         <v>25</v>
       </c>
@@ -3992,7 +3996,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="28">
+    <row r="5" spans="1:4" ht="27">
       <c r="A5" s="4" t="s">
         <v>40</v>
       </c>
@@ -4024,7 +4028,7 @@
       </c>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:4" ht="28">
+    <row r="8" spans="1:4" ht="27">
       <c r="A8" s="2" t="s">
         <v>241</v>
       </c>
@@ -4036,7 +4040,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" ht="42">
+    <row r="9" spans="1:4" ht="40.5">
       <c r="A9" s="4" t="s">
         <v>244</v>
       </c>
@@ -4048,7 +4052,7 @@
       </c>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4" ht="42">
+    <row r="10" spans="1:4" ht="40.5">
       <c r="A10" s="2" t="s">
         <v>247</v>
       </c>
@@ -4060,7 +4064,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" ht="42">
+    <row r="11" spans="1:4" ht="40.5">
       <c r="A11" s="4" t="s">
         <v>250</v>
       </c>
@@ -4072,7 +4076,7 @@
       </c>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" ht="42">
+    <row r="12" spans="1:4" ht="40.5">
       <c r="A12" s="2" t="s">
         <v>253</v>
       </c>
@@ -4084,7 +4088,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" ht="28">
+    <row r="13" spans="1:4" ht="27">
       <c r="A13" s="4" t="s">
         <v>256</v>
       </c>
@@ -4096,7 +4100,7 @@
       </c>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" ht="42">
+    <row r="14" spans="1:4" ht="40.5">
       <c r="A14" s="2" t="s">
         <v>259</v>
       </c>
@@ -4108,7 +4112,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:4" ht="42">
+    <row r="15" spans="1:4" ht="40.5">
       <c r="A15" s="4" t="s">
         <v>262</v>
       </c>
@@ -4120,7 +4124,7 @@
       </c>
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:4" ht="42">
+    <row r="16" spans="1:4" ht="40.5">
       <c r="A16" s="2" t="s">
         <v>265</v>
       </c>
@@ -4132,7 +4136,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" ht="42">
+    <row r="17" spans="1:4" ht="40.5">
       <c r="A17" s="4" t="s">
         <v>268</v>
       </c>
@@ -4153,7 +4157,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -4166,7 +4170,7 @@
     <col min="9" max="9" width="46" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17.5">
+    <row r="1" spans="1:9" ht="18.75">
       <c r="A1" s="16" t="s">
         <v>271</v>
       </c>
@@ -4192,7 +4196,7 @@
       <c r="H2" s="17"/>
       <c r="I2" s="17"/>
     </row>
-    <row r="3" spans="1:9" ht="28">
+    <row r="3" spans="1:9" ht="27">
       <c r="A3" s="1" t="s">
         <v>273</v>
       </c>
@@ -4221,7 +4225,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="28">
+    <row r="4" spans="1:9" ht="27">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -4250,7 +4254,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="28">
+    <row r="5" spans="1:9" ht="27">
       <c r="A5" s="4">
         <v>2</v>
       </c>
@@ -4279,7 +4283,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="42">
+    <row r="6" spans="1:9" ht="40.5">
       <c r="A6" s="2">
         <v>3</v>
       </c>
@@ -4308,7 +4312,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="42">
+    <row r="7" spans="1:9" ht="40.5">
       <c r="A7" s="4">
         <v>4</v>
       </c>
@@ -4337,7 +4341,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="28">
+    <row r="8" spans="1:9" ht="27">
       <c r="A8" s="2">
         <v>5</v>
       </c>
@@ -4366,7 +4370,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="28">
+    <row r="9" spans="1:9" ht="27">
       <c r="A9" s="4">
         <v>6</v>
       </c>
@@ -4482,7 +4486,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="28">
+    <row r="13" spans="1:9" ht="27">
       <c r="A13" s="4">
         <v>10</v>
       </c>
@@ -4540,7 +4544,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="28">
+    <row r="15" spans="1:9" ht="27">
       <c r="A15" s="4">
         <v>12</v>
       </c>
@@ -4569,7 +4573,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="42">
+    <row r="16" spans="1:9" ht="40.5">
       <c r="A16" s="2">
         <v>13</v>
       </c>
@@ -4598,7 +4602,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="28">
+    <row r="17" spans="1:9" ht="27">
       <c r="A17" s="4">
         <v>14</v>
       </c>
@@ -4627,7 +4631,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="28">
+    <row r="18" spans="1:9" ht="27">
       <c r="A18" s="2">
         <v>15</v>
       </c>
@@ -4656,7 +4660,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="28">
+    <row r="19" spans="1:9" ht="27">
       <c r="A19" s="4">
         <v>16</v>
       </c>
@@ -4685,7 +4689,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="28">
+    <row r="20" spans="1:9" ht="27">
       <c r="A20" s="2">
         <v>17</v>
       </c>
@@ -4772,7 +4776,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="28">
+    <row r="23" spans="1:9" ht="27">
       <c r="A23" s="4">
         <v>20</v>
       </c>
@@ -4801,7 +4805,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="28">
+    <row r="24" spans="1:9" ht="27">
       <c r="A24" s="2">
         <v>21</v>
       </c>
@@ -4859,7 +4863,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="28">
+    <row r="26" spans="1:9" ht="27">
       <c r="A26" s="2">
         <v>23</v>
       </c>
@@ -4888,7 +4892,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="28">
+    <row r="27" spans="1:9" ht="27">
       <c r="A27" s="4">
         <v>24</v>
       </c>
@@ -4917,7 +4921,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="28">
+    <row r="28" spans="1:9" ht="27">
       <c r="A28" s="2">
         <v>25</v>
       </c>
@@ -5004,7 +5008,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="28">
+    <row r="31" spans="1:9" ht="27">
       <c r="A31" s="4">
         <v>28</v>
       </c>
@@ -5062,7 +5066,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="28">
+    <row r="33" spans="1:9" ht="27">
       <c r="A33" s="4">
         <v>30</v>
       </c>
@@ -5091,7 +5095,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="28">
+    <row r="34" spans="1:9" ht="27">
       <c r="A34" s="2">
         <v>31</v>
       </c>
@@ -5149,7 +5153,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="28">
+    <row r="36" spans="1:9" ht="27">
       <c r="A36" s="2">
         <v>33</v>
       </c>
@@ -5207,7 +5211,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="28">
+    <row r="38" spans="1:9" ht="27">
       <c r="A38" s="2">
         <v>35</v>
       </c>
@@ -5236,7 +5240,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="28">
+    <row r="39" spans="1:9" ht="27">
       <c r="A39" s="4">
         <v>36</v>
       </c>
@@ -5278,7 +5282,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
@@ -5292,7 +5296,7 @@
     <col min="11" max="11" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.5">
+    <row r="1" spans="1:11" ht="18.75">
       <c r="A1" s="16" t="s">
         <v>404</v>
       </c>
@@ -5322,7 +5326,7 @@
       <c r="J2" s="17"/>
       <c r="K2" s="17"/>
     </row>
-    <row r="3" spans="1:11" ht="28">
+    <row r="3" spans="1:11" ht="27">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -5357,7 +5361,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="70">
+    <row r="4" spans="1:11" ht="67.5">
       <c r="A4" s="2" t="s">
         <v>415</v>
       </c>
@@ -5386,7 +5390,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="56">
+    <row r="5" spans="1:11" ht="54">
       <c r="A5" s="4" t="s">
         <v>38</v>
       </c>
@@ -5413,7 +5417,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="56">
+    <row r="6" spans="1:11" ht="54">
       <c r="A6" s="2" t="s">
         <v>429</v>
       </c>
@@ -5438,7 +5442,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="42">
+    <row r="7" spans="1:11" ht="40.5">
       <c r="A7" s="4" t="s">
         <v>435</v>
       </c>
@@ -5461,7 +5465,7 @@
       <c r="J7" s="5"/>
       <c r="K7" s="4"/>
     </row>
-    <row r="8" spans="1:11" ht="42">
+    <row r="8" spans="1:11" ht="40.5">
       <c r="A8" s="2" t="s">
         <v>439</v>
       </c>
@@ -5488,7 +5492,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="56">
+    <row r="9" spans="1:11" ht="54">
       <c r="A9" s="4" t="s">
         <v>98</v>
       </c>
@@ -5515,7 +5519,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="56">
+    <row r="10" spans="1:11" ht="54">
       <c r="A10" s="2" t="s">
         <v>452</v>
       </c>
@@ -5538,7 +5542,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="42">
+    <row r="11" spans="1:11" ht="40.5">
       <c r="A11" s="4" t="s">
         <v>457</v>
       </c>
@@ -5565,7 +5569,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11" ht="42">
+    <row r="12" spans="1:11" ht="40.5">
       <c r="A12" s="2" t="s">
         <v>463</v>
       </c>
@@ -5590,7 +5594,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="42">
+    <row r="13" spans="1:11" ht="40.5">
       <c r="A13" s="4" t="s">
         <v>142</v>
       </c>
@@ -5615,7 +5619,7 @@
       <c r="J13" s="5"/>
       <c r="K13" s="4"/>
     </row>
-    <row r="14" spans="1:11" ht="42">
+    <row r="14" spans="1:11" ht="40.5">
       <c r="A14" s="2" t="s">
         <v>474</v>
       </c>

</xml_diff>

<commit_message>
Chap 8, Ex 9
</commit_message>
<xml_diff>
--- a/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
+++ b/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_DE2EFB3A9D1E79C6859C80A3377C0E0772D29E3B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF23E7C9-3F0B-47DB-9547-EF99EC340627}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_DE2EFB3A9D1E79C6859C80A3377C0E0772D29E3B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACB6DB31-E324-4919-B6CC-63C6CE377F82}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="481">
   <si>
     <t>Order</t>
   </si>
@@ -1642,6 +1642,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2741,13 +2745,17 @@
       </c>
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="6"/>
+      <c r="L21" s="12">
+        <v>46300</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>232</v>
+      </c>
       <c r="N21" s="6"/>
       <c r="O21" s="6"/>
-      <c r="P21" s="12" t="str">
+      <c r="P21" s="12">
         <f>IF(AND($L21&lt;&gt;"",$M21&lt;&gt;""),$L21+VLOOKUP($M21,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46302</v>
       </c>
       <c r="Q21" s="12"/>
       <c r="R21" s="6"/>
@@ -3696,7 +3704,7 @@
       </c>
       <c r="B7" s="8">
         <f>COUNT('Master Schedule'!L2:L43)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">
@@ -3715,7 +3723,7 @@
       </c>
       <c r="B8" s="8">
         <f ca="1">COUNTIFS('Master Schedule'!P2:P43,"&lt;="&amp;TODAY(),'Master Schedule'!P2:P43,"&gt;0",'Master Schedule'!Q2:Q43,"")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6" t="s">

</xml_diff>

<commit_message>
Chap 8, Ex 9, 31
</commit_message>
<xml_diff>
--- a/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
+++ b/plan/Chapter8_Final_Section_Exercise_Redo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_DE2EFB3A9D1E79C6859C80A3377C0E0772D29E3B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACB6DB31-E324-4919-B6CC-63C6CE377F82}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_4A10487BE2825A7980104F5CE81F24FBE394D2B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CEDB3B7-0C68-4F70-AC99-D7963A926EE6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2385" yWindow="2565" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="481">
   <si>
     <t>Order</t>
   </si>
@@ -330,6 +330,9 @@
     <t>Strengthen pointwise/weak cdf convergence to uniform convergence when the limit is continuous.</t>
   </si>
   <si>
+    <t>Spark</t>
+  </si>
+  <si>
     <t>Ex 9</t>
   </si>
   <si>
@@ -733,9 +736,6 @@
   </si>
   <si>
     <t>Repair the exercise first. Redo next day after rereading the exact theorem/definition; ask for a minimum hint only if still blank.</t>
-  </si>
-  <si>
-    <t>Spark</t>
   </si>
   <si>
     <t>A blurred idea appears but cannot yet carry the proof.</t>
@@ -1642,10 +1642,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2749,7 +2745,7 @@
         <v>46300</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>232</v>
+        <v>97</v>
       </c>
       <c r="N21" s="6"/>
       <c r="O21" s="6"/>
@@ -2775,26 +2771,30 @@
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G22" s="10" t="s">
         <v>33</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J22" s="11"/>
       <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="10"/>
+      <c r="L22" s="11">
+        <v>46301</v>
+      </c>
+      <c r="M22" s="10" t="s">
+        <v>25</v>
+      </c>
       <c r="N22" s="10"/>
       <c r="O22" s="10"/>
-      <c r="P22" s="11" t="str">
+      <c r="P22" s="11">
         <f>IF(AND($L22&lt;&gt;"",$M22&lt;&gt;""),$L22+VLOOKUP($M22,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46303</v>
       </c>
       <c r="Q22" s="11"/>
       <c r="R22" s="10"/>
@@ -2814,26 +2814,30 @@
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J23" s="12"/>
       <c r="K23" s="12"/>
-      <c r="L23" s="12"/>
-      <c r="M23" s="6"/>
+      <c r="L23" s="12">
+        <v>46303</v>
+      </c>
+      <c r="M23" s="6" t="s">
+        <v>25</v>
+      </c>
       <c r="N23" s="6"/>
       <c r="O23" s="6"/>
-      <c r="P23" s="12" t="str">
+      <c r="P23" s="12">
         <f>IF(AND($L23&lt;&gt;"",$M23&lt;&gt;""),$L23+VLOOKUP($M23,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46305</v>
       </c>
       <c r="Q23" s="12"/>
       <c r="R23" s="6"/>
@@ -2848,21 +2852,23 @@
         <v>46295</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I24" s="10"/>
-      <c r="J24" s="11"/>
+      <c r="J24" s="11">
+        <v>46307</v>
+      </c>
       <c r="K24" s="11"/>
       <c r="L24" s="11"/>
       <c r="M24" s="10"/>
@@ -2882,31 +2888,35 @@
         <v>46296</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>94</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J25" s="12"/>
       <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
-      <c r="M25" s="6"/>
+      <c r="L25" s="12">
+        <v>46308</v>
+      </c>
+      <c r="M25" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="N25" s="6"/>
       <c r="O25" s="6"/>
-      <c r="P25" s="12" t="str">
+      <c r="P25" s="12">
         <f>IF(AND($L25&lt;&gt;"",$M25&lt;&gt;""),$L25+VLOOKUP($M25,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46310</v>
       </c>
       <c r="Q25" s="12"/>
       <c r="R25" s="6"/>
@@ -2921,31 +2931,35 @@
         <v>46297</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>94</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J26" s="11"/>
       <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="10"/>
+      <c r="L26" s="11">
+        <v>46309</v>
+      </c>
+      <c r="M26" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="N26" s="10"/>
       <c r="O26" s="10"/>
-      <c r="P26" s="11" t="str">
+      <c r="P26" s="11">
         <f>IF(AND($L26&lt;&gt;"",$M26&lt;&gt;""),$L26+VLOOKUP($M26,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46311</v>
       </c>
       <c r="Q26" s="11"/>
       <c r="R26" s="10"/>
@@ -2960,18 +2974,18 @@
         <v>46298</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
       <c r="H27" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I27" s="6"/>
       <c r="J27" s="12"/>
@@ -2994,21 +3008,21 @@
         <v>46299</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G28" s="10" t="s">
         <v>46</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J28" s="11"/>
       <c r="K28" s="11"/>
@@ -3033,21 +3047,21 @@
         <v>46300</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
       <c r="F29" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>94</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J29" s="12"/>
       <c r="K29" s="12"/>
@@ -3072,21 +3086,21 @@
         <v>46301</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F30" s="10"/>
       <c r="G30" s="10"/>
       <c r="H30" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J30" s="11"/>
       <c r="K30" s="11"/>
@@ -3108,19 +3122,19 @@
         <v>46302</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
       <c r="H31" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
@@ -3142,21 +3156,21 @@
         <v>46303</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J32" s="11"/>
       <c r="K32" s="11"/>
@@ -3178,21 +3192,21 @@
         <v>46304</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
       <c r="F33" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
@@ -3217,21 +3231,21 @@
         <v>46305</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G34" s="10" t="s">
         <v>33</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J34" s="11"/>
       <c r="K34" s="11"/>
@@ -3256,18 +3270,18 @@
         <v>46306</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
       <c r="H35" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I35" s="6"/>
       <c r="J35" s="12"/>
@@ -3290,21 +3304,21 @@
         <v>46307</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D36" s="10"/>
       <c r="E36" s="10"/>
       <c r="F36" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G36" s="10" t="s">
         <v>33</v>
       </c>
       <c r="H36" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J36" s="11"/>
       <c r="K36" s="11"/>
@@ -3329,21 +3343,21 @@
         <v>46308</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
       <c r="F37" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>33</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J37" s="12"/>
       <c r="K37" s="12"/>
@@ -3368,21 +3382,21 @@
         <v>46309</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
       <c r="F38" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J38" s="11"/>
       <c r="K38" s="11"/>
@@ -3407,21 +3421,21 @@
         <v>46310</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
       <c r="F39" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J39" s="12"/>
       <c r="K39" s="12"/>
@@ -3446,19 +3460,19 @@
         <v>46311</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D40" s="10"/>
       <c r="E40" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F40" s="10"/>
       <c r="G40" s="10"/>
       <c r="H40" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J40" s="11"/>
       <c r="K40" s="11"/>
@@ -3480,21 +3494,21 @@
         <v>46312</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
       <c r="H41" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J41" s="12"/>
       <c r="K41" s="12"/>
@@ -3516,19 +3530,19 @@
         <v>46313</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
       <c r="H42" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J42" s="11"/>
       <c r="K42" s="11"/>
@@ -3550,19 +3564,19 @@
         <v>46314</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
       <c r="H43" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J43" s="12"/>
       <c r="K43" s="12"/>
@@ -3584,14 +3598,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" sqref="M2:M43" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="R2:R43" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>"Independent,Still Spark,Still Skeleton,Needs Hint,Parked"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="M2:M43" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="O2:O43" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="O2:O43" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Yes,No,N/A"</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="R2:R43" xr:uid="{00000000-0002-0000-0000-000002000000}">
-      <formula1>"Independent,Still Spark,Still Skeleton,Needs Hint,Parked"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="S2:S43" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Yes,No,Not requested"</formula1>
@@ -3616,7 +3630,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18.75">
       <c r="A1" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -3626,7 +3640,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -3644,25 +3658,25 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27">
       <c r="A5" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B5" s="8">
         <f>COUNTIF('Exercise Map'!F4:F39,"Yes")</f>
@@ -3673,15 +3687,15 @@
         <v>43</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="27">
       <c r="A6" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B6" s="8">
         <f>COUNTIF('Exercise Map'!F4:F39,"No")</f>
@@ -3689,56 +3703,56 @@
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="27">
       <c r="A7" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B7" s="8">
         <f>COUNT('Master Schedule'!L2:L43)</f>
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="27">
       <c r="A8" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B8" s="8">
         <f ca="1">COUNTIFS('Master Schedule'!P2:P43,"&lt;="&amp;TODAY(),'Master Schedule'!P2:P43,"&gt;0",'Master Schedule'!Q2:Q43,"")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6" t="s">
         <v>32</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="27">
       <c r="A9" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B9" s="8">
         <f>COUNT('Section Plan'!J4:J14)</f>
@@ -3746,13 +3760,13 @@
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>27</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -3773,7 +3787,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="15" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
@@ -3783,13 +3797,13 @@
     </row>
     <row r="13" spans="1:6" ht="27">
       <c r="A13" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -3797,13 +3811,13 @@
     </row>
     <row r="14" spans="1:6" ht="27">
       <c r="A14" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -3811,13 +3825,13 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
@@ -3825,13 +3839,13 @@
     </row>
     <row r="16" spans="1:6" ht="40.5">
       <c r="A16" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
@@ -3839,13 +3853,13 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
@@ -3853,13 +3867,13 @@
     </row>
     <row r="18" spans="1:6" ht="27">
       <c r="A18" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
@@ -3875,7 +3889,7 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="15" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
@@ -3888,10 +3902,10 @@
         <v>32</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
@@ -3899,13 +3913,13 @@
     </row>
     <row r="22" spans="1:6" ht="40.5">
       <c r="A22" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
@@ -3913,13 +3927,13 @@
     </row>
     <row r="23" spans="1:6" ht="27">
       <c r="A23" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
@@ -3950,27 +3964,27 @@
   <sheetData>
     <row r="1" spans="1:4" ht="27">
       <c r="A1" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="40.5">
       <c r="A2" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -3978,7 +3992,7 @@
     </row>
     <row r="3" spans="1:4" ht="27">
       <c r="A3" s="4" t="s">
-        <v>232</v>
+        <v>97</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>233</v>
@@ -4029,7 +4043,7 @@
         <v>239</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>240</v>
@@ -4644,7 +4658,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>321</v>
@@ -4673,7 +4687,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>340</v>
@@ -4963,7 +4977,7 @@
         <v>26</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>371</v>
@@ -4992,7 +5006,7 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>340</v>
@@ -5050,7 +5064,7 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>321</v>
@@ -5502,7 +5516,7 @@
     </row>
     <row r="9" spans="1:11" ht="54">
       <c r="A9" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>446</v>
@@ -5561,7 +5575,7 @@
         <v>459</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>460</v>
@@ -5604,7 +5618,7 @@
     </row>
     <row r="13" spans="1:11" ht="40.5">
       <c r="A13" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>469</v>

</xml_diff>